<commit_message>
auto update pricing 2026-10-28
</commit_message>
<xml_diff>
--- a/llm_pricing.xlsx
+++ b/llm_pricing.xlsx
@@ -525,7 +525,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>国内外主流大模型 API 定价对比（含代理折扣）</t>
+          <t>国内外主流大模型 API 定价对比（含折扣）</t>
         </is>
       </c>
     </row>
@@ -7250,17 +7250,17 @@
       </c>
       <c r="J30" s="8" t="inlineStr">
         <is>
-          <t>6折</t>
+          <t>8.5折</t>
         </is>
       </c>
       <c r="K30" s="9" t="inlineStr">
         <is>
-          <t>¥7.2</t>
+          <t>¥10.2</t>
         </is>
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>¥21.6</t>
+          <t>¥30.6</t>
         </is>
       </c>
       <c r="M30" s="7" t="inlineStr">
@@ -7322,17 +7322,17 @@
       </c>
       <c r="J31" s="8" t="inlineStr">
         <is>
-          <t>4.5折</t>
+          <t>8.5折</t>
         </is>
       </c>
       <c r="K31" s="9" t="inlineStr">
         <is>
-          <t>¥0.36</t>
+          <t>¥0.68</t>
         </is>
       </c>
       <c r="L31" s="9" t="inlineStr">
         <is>
-          <t>¥1.215</t>
+          <t>¥2.295</t>
         </is>
       </c>
       <c r="M31" s="10" t="inlineStr">
@@ -15721,17 +15721,17 @@
       </c>
       <c r="I2" s="8" t="inlineStr">
         <is>
-          <t>6折</t>
+          <t>8.5折</t>
         </is>
       </c>
       <c r="J2" s="9" t="inlineStr">
         <is>
-          <t>¥7.2</t>
+          <t>¥10.2</t>
         </is>
       </c>
       <c r="K2" s="9" t="inlineStr">
         <is>
-          <t>¥21.6</t>
+          <t>¥30.6</t>
         </is>
       </c>
       <c r="L2" s="7" t="inlineStr">
@@ -15788,17 +15788,17 @@
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
-          <t>4.5折</t>
+          <t>8.5折</t>
         </is>
       </c>
       <c r="J3" s="9" t="inlineStr">
         <is>
-          <t>¥0.36</t>
+          <t>¥0.68</t>
         </is>
       </c>
       <c r="K3" s="9" t="inlineStr">
         <is>
-          <t>¥1.215</t>
+          <t>¥2.295</t>
         </is>
       </c>
       <c r="L3" s="10" t="inlineStr">

</xml_diff>